<commit_message>
#32 IOT Button eSpark and Client BOM updated
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.3/BOM/Client BOM IoT-Button v1.3.xlsx
+++ b/Design Files/IoT-Button-v1.3/BOM/Client BOM IoT-Button v1.3.xlsx
@@ -1050,6 +1050,12 @@
     <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1058,12 +1064,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1433,11 +1433,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1475,7 +1475,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="60"/>
+      <c r="M3" s="62"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1494,7 +1494,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="56"/>
-      <c r="M4" s="61"/>
+      <c r="M4" s="63"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1513,7 +1513,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="56"/>
-      <c r="M5" s="61"/>
+      <c r="M5" s="63"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1528,7 +1528,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="56"/>
-      <c r="M6" s="61"/>
+      <c r="M6" s="63"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1543,7 +1543,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="61"/>
+      <c r="M7" s="63"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1558,7 +1558,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="61"/>
+      <c r="M8" s="63"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2637,7 +2637,7 @@
       <c r="L37" s="36">
         <v>1</v>
       </c>
-      <c r="M37" s="62"/>
+      <c r="M37" s="59"/>
     </row>
     <row r="38" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
@@ -2675,7 +2675,7 @@
       <c r="L38" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="M38" s="63" t="s">
+      <c r="M38" s="60" t="s">
         <v>161</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Minor correction in Button BOM #32
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.3/BOM/Client BOM IoT-Button v1.3.xlsx
+++ b/Design Files/IoT-Button-v1.3/BOM/Client BOM IoT-Button v1.3.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Button-v1.3\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\smartmasjid-hardware\Design Files\IoT-Button-v1.3\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
@@ -510,7 +510,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -1109,7 +1109,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1631,7 +1631,7 @@
         <v>6</v>
       </c>
       <c r="L10" s="36">
-        <f t="shared" ref="L10:L35" si="0">K10*5</f>
+        <f t="shared" ref="L10:L36" si="0">K10*5</f>
         <v>30</v>
       </c>
       <c r="M10" s="36"/>
@@ -2597,7 +2597,8 @@
         <v>1</v>
       </c>
       <c r="L36" s="36">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="M36" s="36"/>
     </row>

</xml_diff>

<commit_message>
#32 Screw added in Client and eSpark BOM
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.3/BOM/Client BOM IoT-Button v1.3.xlsx
+++ b/Design Files/IoT-Button-v1.3/BOM/Client BOM IoT-Button v1.3.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\smartmasjid-hardware\Design Files\IoT-Button-v1.3\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Button-v1.3\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="166">
   <si>
     <t>Component list</t>
   </si>
@@ -498,19 +498,31 @@
     <t>Screws</t>
   </si>
   <si>
-    <t>(M2 Screw Lentgh 4mm), (M2 Screw Lentgh 5mm), (M2 Screw Lentgh 6mm)</t>
-  </si>
-  <si>
     <t>Tinde</t>
   </si>
   <si>
-    <t>Multiple Lentgh Screw Required</t>
+    <t>M2 (4mm)</t>
+  </si>
+  <si>
+    <t>M2 (5mm)</t>
+  </si>
+  <si>
+    <t>M2 (6mm)</t>
+  </si>
+  <si>
+    <t>(M2 Screw thread  length 4mm)</t>
+  </si>
+  <si>
+    <t>(M2 Screw thread Lentgh 5mm)</t>
+  </si>
+  <si>
+    <t>(M2 Screw Thread Lentgh 6mm)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -695,7 +707,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -890,12 +902,99 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1053,8 +1152,33 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1064,6 +1188,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1109,7 +1251,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1407,7 +1549,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1418,7 +1560,7 @@
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.140625" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.7109375" customWidth="1"/>
     <col min="13" max="13" width="29.42578125" customWidth="1"/>
@@ -1433,11 +1575,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1475,7 +1617,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="62"/>
+      <c r="M3" s="71"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1494,7 +1636,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="56"/>
-      <c r="M4" s="63"/>
+      <c r="M4" s="72"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1513,7 +1655,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="56"/>
-      <c r="M5" s="63"/>
+      <c r="M5" s="72"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1528,7 +1670,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="56"/>
-      <c r="M6" s="63"/>
+      <c r="M6" s="72"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1543,7 +1685,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="63"/>
+      <c r="M7" s="72"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1558,7 +1700,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="63"/>
+      <c r="M8" s="72"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1631,7 +1773,7 @@
         <v>6</v>
       </c>
       <c r="L10" s="36">
-        <f t="shared" ref="L10:L36" si="0">K10*5</f>
+        <f t="shared" ref="L10:L40" si="0">K10*5</f>
         <v>30</v>
       </c>
       <c r="M10" s="36"/>
@@ -2527,7 +2669,7 @@
     <row r="35" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="50">
-        <f t="shared" ref="B35:B38" si="2">ROW(B35) - ROW($B$9)</f>
+        <f t="shared" ref="B35:B40" si="2">ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
       <c r="C35" s="57" t="s">
@@ -2630,7 +2772,7 @@
         <v>145</v>
       </c>
       <c r="J37" s="58" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K37" s="36">
         <v>1</v>
@@ -2640,89 +2782,162 @@
       </c>
       <c r="M37" s="59"/>
     </row>
-    <row r="38" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="50">
         <f t="shared" si="2"/>
         <v>29</v>
       </c>
-      <c r="C38" s="57" t="s">
+      <c r="C38" s="73" t="s">
         <v>158</v>
       </c>
-      <c r="D38" s="36" t="s">
+      <c r="D38" s="76" t="s">
         <v>150</v>
       </c>
-      <c r="E38" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="F38" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="G38" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="H38" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="I38" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="J38" s="58" t="s">
+      <c r="E38" s="66" t="s">
+        <v>163</v>
+      </c>
+      <c r="F38" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="G38" s="67" t="s">
+        <v>160</v>
+      </c>
+      <c r="H38" s="68" t="s">
+        <v>145</v>
+      </c>
+      <c r="I38" s="69" t="s">
+        <v>145</v>
+      </c>
+      <c r="J38" s="62" t="s">
         <v>152</v>
       </c>
-      <c r="K38" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="L38" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="M38" s="60" t="s">
+      <c r="K38" s="36">
+        <v>3</v>
+      </c>
+      <c r="L38" s="36">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="M38" s="65"/>
+    </row>
+    <row r="39" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1"/>
+      <c r="B39" s="50">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="C39" s="74"/>
+      <c r="D39" s="77"/>
+      <c r="E39" s="66" t="s">
+        <v>164</v>
+      </c>
+      <c r="F39" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="G39" s="67" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A39" s="1"/>
-      <c r="B39" s="31"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="34"/>
-      <c r="G39" s="35"/>
-      <c r="H39" s="34"/>
-      <c r="I39" s="35"/>
-      <c r="J39" s="35"/>
-      <c r="K39" s="35"/>
-      <c r="L39" s="35"/>
-      <c r="M39" s="41"/>
+      <c r="H39" s="68" t="s">
+        <v>145</v>
+      </c>
+      <c r="I39" s="69" t="s">
+        <v>145</v>
+      </c>
+      <c r="J39" s="63" t="s">
+        <v>152</v>
+      </c>
+      <c r="K39" s="36">
+        <v>2</v>
+      </c>
+      <c r="L39" s="36">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="M39" s="60"/>
     </row>
     <row r="40" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="24"/>
-      <c r="C40" s="49"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="9"/>
-      <c r="I40" s="9"/>
-      <c r="J40" s="9"/>
-      <c r="K40" s="9"/>
-      <c r="L40" s="9"/>
-      <c r="M40" s="42"/>
+      <c r="B40" s="50">
+        <f t="shared" si="2"/>
+        <v>31</v>
+      </c>
+      <c r="C40" s="75"/>
+      <c r="D40" s="78"/>
+      <c r="E40" s="66" t="s">
+        <v>165</v>
+      </c>
+      <c r="F40" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="G40" s="67" t="s">
+        <v>162</v>
+      </c>
+      <c r="H40" s="68" t="s">
+        <v>145</v>
+      </c>
+      <c r="I40" s="69" t="s">
+        <v>145</v>
+      </c>
+      <c r="J40" s="64" t="s">
+        <v>152</v>
+      </c>
+      <c r="K40" s="36">
+        <v>4</v>
+      </c>
+      <c r="L40" s="36">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="M40" s="60"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A41" s="1"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="35"/>
+      <c r="H41" s="34"/>
+      <c r="I41" s="35"/>
+      <c r="J41" s="61"/>
+      <c r="K41" s="35"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="41"/>
+    </row>
+    <row r="42" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="49"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
+      <c r="J42" s="9"/>
+      <c r="K42" s="9"/>
+      <c r="L42" s="9"/>
+      <c r="M42" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="I1:M1"/>
     <mergeCell ref="M3:M8"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="D38:D40"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="J35" r:id="rId1"/>
     <hyperlink ref="J36" r:id="rId2"/>
     <hyperlink ref="J37" r:id="rId3"/>
     <hyperlink ref="J38" r:id="rId4"/>
+    <hyperlink ref="J40" r:id="rId5"/>
+    <hyperlink ref="J39" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
-  <drawing r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>